<commit_message>
chore: Dong bo toan bo du lieu Master Data, Excel Book1.xlsx va phan he Can Lua
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -550,7 +550,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="77" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
@@ -755,7 +755,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N579"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -40127,7 +40127,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -41584,7 +41584,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -41784,7 +41784,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -42019,7 +42019,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>

</xml_diff>